<commit_message>
feat(ideias): artigos do LinkedIn entram na lista
19 textos do LinkedIn (2015–2020) entram como link externo, com título,
data e link. Cópias de textos que já estão na lista ficam de fora e
viram observação na planilha; as versões em inglês de "Em tempos de
crise" e "Empreender empreendedores" e o par PT/EN de "99 motivos"
entram como Título/URL em inglês.

Na /en/ideas, quando a versão em inglês está noutro veículo, a linha
mostra o veículo de destino (NeoFeed → Substack, Blog → LinkedIn).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ideias.xlsx
+++ b/data/ideias.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -568,8 +568,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="b">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -610,13 +612,15 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Estava na Na mídia como texto assinado.</t>
+          <t>Estava na Na mídia como texto assinado. Também no LinkedIn em 2026-06-22.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="b">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -662,8 +666,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="b">
-        <v>1</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -701,8 +707,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="b">
-        <v>1</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -736,148 +744,156 @@
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="b">
-        <v>1</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2019-01-12</t>
+          <t>2020-11-23</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>President Bolsonaro should boost Brazil’s entrepreneurial ecosystem</t>
+          <t>Como as cleantechs estão transformando o mundo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TechCrunch</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2019/01/12/president-bolsonaro-should-boost-brazils-entrepreneurial-ecosystem</t>
+          <t>https://www.linkedin.com/pulse/como-cleantechs-est%C3%A3o-transformando-o-mundo-romero-rodrigues</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Estava na Na mídia como texto assinado.</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
-        <v>1</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2017-05-13</t>
+          <t>2020-10-02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Brazil’s fintech boom offers new vertical opportunities for investors</t>
+          <t>Eureka! Eureka!</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TechCrunch</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2017/05/13/brazils-fintech-boom-offers-new-vertical-opportunities-for-investors</t>
+          <t>https://www.linkedin.com/pulse/eureka-romero-rodrigues</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Estava na Na mídia como texto assinado.</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
-        <v>1</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2016-09-17</t>
+          <t>2020-07-29</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Brazil’s tech-sector bright spots beckon as it begins to emerge from long economic crisis</t>
+          <t>Startups são o passaporte para o "velho novo normal"</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TechCrunch</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2016/09/17/brazils-tech-sector-bright-spots-beckon-as-it-begins-to-emerge-from-long-economic-crisis</t>
+          <t>https://www.linkedin.com/pulse/startups-s%C3%A3o-o-passaporte-para-velho-novo-normal-romero-rodrigues</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Estava na Na mídia como texto assinado.</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="b">
-        <v>1</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2016-07-01</t>
+          <t>2020-06-10</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Porque a ineficiência crônica da América Latina é uma fossa competitiva para o segmento de O2O no mobile brasileiro</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>disrupcao-mobilidade</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>disrupcao-mobilidade.md</t>
-        </is>
-      </c>
+          <t>Como vai a saúde mental do seu time?</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/como-vai-sa%C3%BAde-mental-do-seu-time-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>pt</t>
@@ -887,75 +903,79 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
-        <v>1</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2016-06-25</t>
+          <t>2020-05-26</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Latin America’s chronic inefficiency could drive more O2O commerce growth</t>
+          <t>Nossos relacionamentos definirão os negócios de sucesso pós-pandemia</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>TechCrunch</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2016/06/25/latin-americas-chronic-inefficiency-could-drive-more-o2o-commerce-growth</t>
+          <t>https://www.linkedin.com/pulse/rela%C3%A7%C3%B5es-reconfiguradas-perspectivas-do-venture-para-o-rodrigues</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Estava na Na mídia como texto assinado.</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
-        <v>1</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2016-06-07</t>
+          <t>2020-01-16</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>6 influenciadores para seguir nas redes (e o que aprender com eles)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>6-influenciadores-para-seguir-nas-redes-e-o-que-aprender-com-eles</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>6-influenciadores-para-seguir-nas-redes-e-o-que-aprender-com-eles.md</t>
-        </is>
-      </c>
+          <t>Vida de Startup: O que é venture capital?</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/vida-de-startup-o-que-%C3%A9-venture-capital-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>pt</t>
@@ -965,75 +985,79 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
-        <v>1</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2015-11-27</t>
+          <t>2019-01-12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Escrevendo um Business Plan</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>escrevendo-um-business-plan</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>escrevendo-um-business-plan.md</t>
-        </is>
-      </c>
+          <t>President Bolsonaro should boost Brazil’s entrepreneurial ecosystem</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2019/01/12/president-bolsonaro-should-boost-brazils-entrepreneurial-ecosystem</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Estava na Na mídia como texto assinado.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
-        <v>1</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2015-11-11</t>
+          <t>2018-12-06</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Empreender empreendedores, meu próximo capítulo</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>empreender-empreendedores-meu-proximo-capitulo</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>empreender-empreendedores-meu-proximo-capitulo.md</t>
-        </is>
-      </c>
+          <t>Repassa é a mais nova investida da Redpoint eventures</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/repassa-%C3%A9-mais-nova-investida-da-redpoint-eventures-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1043,36 +1067,38 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
-        <v>1</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2015-11-05</t>
+          <t>2018-10-09</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>São Paulo Tech Week acontece na cidade</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>sao-paulo-tech-week-vai-ate-segunda</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>sao-paulo-tech-week-vai-ate-segunda.md</t>
-        </is>
-      </c>
+          <t>#amorsim</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/amorsim-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1082,75 +1108,87 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2015-09-15</t>
+          <t>2018-01-10</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Movimento Compre do Pequeno</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>movimento-compre-do-pequeno</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>movimento-compre-do-pequeno.md</t>
-        </is>
-      </c>
+          <t>99 (ou 1 bilhão de) motivos para ficar (ainda mais) otimista com tecnologia em 2018</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/99-ou-1-bilh%C3%A3o-de-motivos-para-ficar-ainda-mais-com-em-rodrigues</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>pt</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>99 (or 1 billion) reasons to stay (even more) optimistic about tech in 2018</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/99-1-billion-reasons-stay-even-more-optimistic-tech-2018-rodrigues</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse. Versão em inglês de 2018-01-23.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2015-08-28</t>
+          <t>2017-09-25</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Seu negócio está pronto para o “homo mobilis”?</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>seu-negocio-esta-pronto-para-o-homo-mobilis</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>seu-negocio-esta-pronto-para-o-homo-mobilis.md</t>
-        </is>
-      </c>
+          <t>Empreendedores e suas bolinhas de gude</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/empreendedores-e-suas-bolinhas-de-gude-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1160,36 +1198,38 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="b">
-        <v>1</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2015-08-05</t>
+          <t>2017-08-23</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Em tempos de crise, start it up!</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>em-tempos-de-crise-start-it-up</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>em-tempos-de-crise-start-it-up.md</t>
-        </is>
-      </c>
+          <t>Cubo ao quadrado!</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/cubo-ao-quadrado-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1199,36 +1239,38 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="b">
-        <v>1</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2015-07-07</t>
+          <t>2017-06-29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sem crise, empreendedor</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>sem-crise-empreendedor</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>sem-crise-empreendedor.md</t>
-        </is>
-      </c>
+          <t>Boom de fintechs brasileiras oferece novas oportunidades para os investidores</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/boom-de-fintechs-brasileiras-oferece-novas-para-os-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1238,75 +1280,79 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse. Versão em português do texto do TechCrunch de 2017-05-13.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="b">
-        <v>1</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2015-06-23</t>
+          <t>2017-05-13</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5 lições de liderança que você pode aprender com Game of Thrones</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>5-licoes-de-lideranca-que-voce-pode-aprender-com-game-of-thrones</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>5-licoes-de-lideranca-que-voce-pode-aprender-com-game-of-thrones.md</t>
-        </is>
-      </c>
+          <t>Brazil’s fintech boom offers new vertical opportunities for investors</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2017/05/13/brazils-fintech-boom-offers-new-vertical-opportunities-for-investors</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Estava na Na mídia como texto assinado.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="b">
-        <v>1</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2015-06-18</t>
+          <t>2016-12-28</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>8 dicas para você melhorar pessoal e profissionalmente</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>8-dicas-para-voce-melhorar-pessoal-e-profissionalmente</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>8-dicas-para-voce-melhorar-pessoal-e-profissionalmente.md</t>
-        </is>
-      </c>
+          <t>Alguém sabe a cor da atitude pra usar no Réveillon?</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/algu%C3%A9m-sabe-cor-da-atitude-pra-usar-r%C3%A9veillon-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1316,36 +1362,38 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="b">
-        <v>1</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2015-06-12</t>
+          <t>2016-11-07</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>5 dicas valiosas do homem mais rico do Brasil</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>5-dicas-valiosas-do-homem-mais-rico-do-brasil</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>5-dicas-valiosas-do-homem-mais-rico-do-brasil.md</t>
-        </is>
-      </c>
+          <t>Forças do setor de tecnologia do Brasil acenam e começam a emergir da longa crise econômica</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/for%C3%A7as-do-setor-de-tecnologia-brasil-acenam-e-come%C3%A7am-rodrigues</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1355,73 +1403,77 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse. Versão em português do texto do TechCrunch de 2016-09-17.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="b">
-        <v>1</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2015-05-25</t>
+          <t>2016-09-17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>5 lições empreendedoras de um dos maiores fotógrafos brasileiros</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>5-licoes-empreendedoras-de-um-dos-maiores-fotografos-brasileiros</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>5-licoes-empreendedoras-de-um-dos-maiores-fotografos-brasileiros.md</t>
-        </is>
-      </c>
+          <t>Brazil’s tech-sector bright spots beckon as it begins to emerge from long economic crisis</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2016/09/17/brazils-tech-sector-bright-spots-beckon-as-it-begins-to-emerge-from-long-economic-crisis</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Estava na Na mídia como texto assinado.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="b">
-        <v>1</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>2015-05-06</t>
+          <t>2016-07-01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>15 guias grátis para educar o profissional de e-commerce</t>
+          <t>Porque a ineficiência crônica da América Latina é uma fossa competitiva para o segmento de O2O no mobile brasileiro</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>15-guias-gratis-de-e-commerce</t>
+          <t>disrupcao-mobilidade</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>15-guias-gratis-de-e-commerce.md</t>
+          <t>disrupcao-mobilidade.md</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1433,73 +1485,77 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Recuperado do blog antigo (Wayback Machine). Também no LinkedIn em 2016-06-29.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="b">
-        <v>1</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2015-04-16</t>
+          <t>2016-06-25</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Quem é seu mentor?</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>quem-e-seu-mentor</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>quem-e-seu-mentor.md</t>
-        </is>
-      </c>
+          <t>Latin America’s chronic inefficiency could drive more O2O commerce growth</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2016/06/25/latin-americas-chronic-inefficiency-could-drive-more-o2o-commerce-growth</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>en</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Estava na Na mídia como texto assinado.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="b">
-        <v>1</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>2015-02-26</t>
+          <t>2016-06-07</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Qual é a estratégia para o m-commerce?</t>
+          <t>6 influenciadores para seguir nas redes (e o que aprender com eles)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>qual-e-a-estrategia-para-o-m-commerce</t>
+          <t>6-influenciadores-para-seguir-nas-redes-e-o-que-aprender-com-eles</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>qual-e-a-estrategia-para-o-m-commerce.md</t>
+          <t>6-influenciadores-para-seguir-nas-redes-e-o-que-aprender-com-eles.md</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1516,31 +1572,33 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="b">
-        <v>1</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2015-02-10</t>
+          <t>2016-05-04</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4 dicas de comediantes para melhorar sua fala em público</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>4-dicas-de-comediantes-para-falar-em-publico</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>4-dicas-de-comediantes-para-falar-em-publico.md</t>
-        </is>
-      </c>
+          <t>Está na hora de rever seus conceitos de concorrência</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/est%C3%A1-na-hora-de-rever-seus-conceitos-concorr%C3%AAncia-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1550,36 +1608,38 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="b">
-        <v>1</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>2015-02-06</t>
+          <t>2015-12-18</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Divulgado o relatório mais completo sobre o E-commerce Brasileiro em 2014</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>relatorio-completo-sobre-o-e-commerce</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>relatorio-completo-sobre-o-e-commerce.md</t>
-        </is>
-      </c>
+          <t>A ‘produtificação’ dos serviços</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/produtifica%C3%A7%C3%A3o-dos-servi%C3%A7os-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1589,34 +1649,36 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="b">
-        <v>1</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2015-02-03</t>
+          <t>2015-11-27</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>5 dicas de liderança de Abraham Lincoln</t>
+          <t>Escrevendo um Business Plan</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>5-dicas-de-lideranca-de-abraham-lincoln</t>
+          <t>escrevendo-um-business-plan</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>5-dicas-de-lideranca-de-abraham-lincoln.md</t>
+          <t>escrevendo-um-business-plan.md</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1633,29 +1695,31 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="b">
-        <v>1</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>2015-01-19</t>
+          <t>2015-11-11</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Por que Anjo?</t>
+          <t>Empreender empreendedores, meu próximo capítulo</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>por-que-anjo</t>
+          <t>empreender-empreendedores-meu-proximo-capitulo</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>por-que-anjo.md</t>
+          <t>empreender-empreendedores-meu-proximo-capitulo.md</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1663,40 +1727,50 @@
           <t>pt</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Undertaking my next chapter with Redpoint eventures</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/undertaking-my-next-chapter-redpoint-eventures-romero-rodrigues</t>
+        </is>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Recuperado do blog antigo (Wayback Machine). Também no LinkedIn (PT e EN, 2015-11-11).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="b">
-        <v>1</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2015-01-07</t>
+          <t>2015-11-05</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Empreender é a arte da superação</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>empreender-e-a-arte-da-superacao</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>empreender-e-a-arte-da-superacao.md</t>
-        </is>
-      </c>
+          <t>Os números que não veem crise</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/os-n%C3%BAmeros-que-n%C3%A3o-veem-crise-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1706,34 +1780,36 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="b">
-        <v>1</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>2014-12-01</t>
+          <t>2015-11-05</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Black Friday 2014 movimenta 1,16 bilhão</t>
+          <t>São Paulo Tech Week acontece na cidade</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>black-friday-2014-movimenta-116-bilhao-na-black-friday</t>
+          <t>sao-paulo-tech-week-vai-ate-segunda</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>black-friday-2014-movimenta-116-bilhao-na-black-friday.md</t>
+          <t>sao-paulo-tech-week-vai-ate-segunda.md</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1750,31 +1826,33 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="b">
-        <v>1</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2014-11-24</t>
+          <t>2015-09-17</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Por um choque de inovação no Poder Público</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>por-um-choque-de-inovacao-no-poder-publico</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>por-um-choque-de-inovacao-no-poder-publico.md</t>
-        </is>
-      </c>
+          <t>Hora de virar a página. Mas não de terminar o livro</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/hora-de-virar-p%C3%A1gina-mas-n%C3%A3o-terminar-o-livro-romero-rodrigues</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>pt</t>
@@ -1784,34 +1862,36 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>LinkedIn Pulse.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="b">
-        <v>1</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>2014-11-13</t>
+          <t>2015-09-15</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Investidor-anjo ou diabo?</t>
+          <t>Movimento Compre do Pequeno</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>investidor-anjo-ou-diabo</t>
+          <t>movimento-compre-do-pequeno</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>investidor-anjo-ou-diabo.md</t>
+          <t>movimento-compre-do-pequeno.md</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1828,29 +1908,31 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="b">
-        <v>1</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2014-10-15</t>
+          <t>2015-08-28</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>E o empreendedorismo, candidatos?</t>
+          <t>Seu negócio está pronto para o “homo mobilis”?</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>e-o-empreendedorismo</t>
+          <t>seu-negocio-esta-pronto-para-o-homo-mobilis</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>e-o-empreendedorismo.md</t>
+          <t>seu-negocio-esta-pronto-para-o-homo-mobilis.md</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1862,34 +1944,36 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Recuperado do blog antigo (Wayback Machine). Também no LinkedIn em 2015-08-25, com o título 'Dados surpreendentes sobre e-commerce no celular mostram caminho para atravessar a crise'.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="b">
-        <v>1</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2014-09-16</t>
+          <t>2015-08-05</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Seu concorrente está a um dedo de distância</t>
+          <t>Em tempos de crise, start it up!</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>mobilidade-seu-concorrente-esta-a-um-dedo-de-distancia</t>
+          <t>em-tempos-de-crise-start-it-up</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>mobilidade-seu-concorrente-esta-a-um-dedo-de-distancia.md</t>
+          <t>em-tempos-de-crise-start-it-up.md</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1897,38 +1981,48 @@
           <t>pt</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>There’s an opportunity in Brazil to innovate and reinvent old industries as new again</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/theres-opportunity-brazil-innovate-reinvent-old-new-again-rodrigues</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Recuperado do blog antigo (Wayback Machine).</t>
+          <t>Recuperado do blog antigo (Wayback Machine). Também no LinkedIn (PT e EN, 2015-09-11).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="b">
-        <v>1</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2014-08-14</t>
+          <t>2015-07-07</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Acredite no impossível! Palestra na Feira do Empreendedor Sebrae</t>
+          <t>Sem crise, empreendedor</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>palestra-na-feira-do-empreendedor-sebrae</t>
+          <t>sem-crise-empreendedor</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>palestra-na-feira-do-empreendedor-sebrae.md</t>
+          <t>sem-crise-empreendedor.md</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1945,29 +2039,31 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="b">
-        <v>1</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2014-07-28</t>
+          <t>2015-06-23</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10 dicas para você conseguir um bom investidor-anjo</t>
+          <t>5 lições de liderança que você pode aprender com Game of Thrones</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>10-dicas-para-voce-conseguir-um-bom-investidor-anjo</t>
+          <t>5-licoes-de-lideranca-que-voce-pode-aprender-com-game-of-thrones</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>10-dicas-para-voce-conseguir-um-bom-investidor-anjo.md</t>
+          <t>5-licoes-de-lideranca-que-voce-pode-aprender-com-game-of-thrones.md</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1984,29 +2080,31 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="b">
-        <v>1</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2014-06-06</t>
+          <t>2015-06-18</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Reflexões de um debutante</t>
+          <t>8 dicas para você melhorar pessoal e profissionalmente</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>reflexoes-de-um-debutante</t>
+          <t>8-dicas-para-voce-melhorar-pessoal-e-profissionalmente</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>reflexoes-de-um-debutante.md</t>
+          <t>8-dicas-para-voce-melhorar-pessoal-e-profissionalmente.md</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2023,29 +2121,31 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="b">
-        <v>1</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>2014-04-22</t>
+          <t>2015-06-12</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Manual para um E-commerce B2B de Sucesso</t>
+          <t>5 dicas valiosas do homem mais rico do Brasil</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>manual-para-um-e-commerce-b2b-de-sucesso</t>
+          <t>5-dicas-valiosas-do-homem-mais-rico-do-brasil</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>manual-para-um-e-commerce-b2b-de-sucesso.md</t>
+          <t>5-dicas-valiosas-do-homem-mais-rico-do-brasil.md</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2062,29 +2162,31 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="b">
-        <v>1</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2014-03-28</t>
+          <t>2015-05-25</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Tendências para a tecnologia em 2014</t>
+          <t>5 lições empreendedoras de um dos maiores fotógrafos brasileiros</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>tendencias-para-a-tecnologia-em-2014</t>
+          <t>5-licoes-empreendedoras-de-um-dos-maiores-fotografos-brasileiros</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>tendencias-para-a-tecnologia-em-2014.md</t>
+          <t>5-licoes-empreendedoras-de-um-dos-maiores-fotografos-brasileiros.md</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2101,29 +2203,31 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="b">
-        <v>1</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>2014-02-06</t>
+          <t>2015-05-06</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Como usar as redes sociais para atrair talentos para a sua startup</t>
+          <t>15 guias grátis para educar o profissional de e-commerce</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>como-usar-as-redes-sociais-para-atrair-talentos-para-a-sua-startup</t>
+          <t>15-guias-gratis-de-e-commerce</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>como-usar-as-redes-sociais-para-atrair-talentos-para-a-sua-startup.md</t>
+          <t>15-guias-gratis-de-e-commerce.md</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2140,29 +2244,31 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="b">
-        <v>1</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2014-01-28</t>
+          <t>2015-04-16</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Um legado para gestão startup</t>
+          <t>Quem é seu mentor?</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>um-legado-para-gestao-startup</t>
+          <t>quem-e-seu-mentor</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>um-legado-para-gestao-startup.md</t>
+          <t>quem-e-seu-mentor.md</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2179,29 +2285,31 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="b">
-        <v>1</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2014-01-10</t>
+          <t>2015-02-26</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Seis dicas para melhorar o perfil no LinkedIn</t>
+          <t>Qual é a estratégia para o m-commerce?</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>seis-dicas-para-melhorar-o-perfil-no-linkedin</t>
+          <t>qual-e-a-estrategia-para-o-m-commerce</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>seis-dicas-para-melhorar-o-perfil-no-linkedin.md</t>
+          <t>qual-e-a-estrategia-para-o-m-commerce.md</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2218,29 +2326,31 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="b">
-        <v>1</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2013-11-14</t>
+          <t>2015-02-10</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Marco Civil, sociedade e mercado digital</t>
+          <t>4 dicas de comediantes para melhorar sua fala em público</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>marco-civil-sociedade-e-mercado-digital</t>
+          <t>4-dicas-de-comediantes-para-falar-em-publico</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>marco-civil-sociedade-e-mercado-digital.md</t>
+          <t>4-dicas-de-comediantes-para-falar-em-publico.md</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2257,29 +2367,31 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="b">
-        <v>1</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2013-11-07</t>
+          <t>2015-02-06</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Uma história de sucesso: de uma garagem na Pedroso Alvarenga para o mundo</t>
+          <t>Divulgado o relatório mais completo sobre o E-commerce Brasileiro em 2014</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>uma-historia-de-sucesso</t>
+          <t>relatorio-completo-sobre-o-e-commerce</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>uma-historia-de-sucesso.md</t>
+          <t>relatorio-completo-sobre-o-e-commerce.md</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2296,29 +2408,31 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="b">
-        <v>1</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2013-09-13</t>
+          <t>2015-02-03</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>A Cultura do Fracasso</t>
+          <t>5 dicas de liderança de Abraham Lincoln</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>a-cultura-do-fracasso</t>
+          <t>5-dicas-de-lideranca-de-abraham-lincoln</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>a-cultura-do-fracasso.md</t>
+          <t>5-dicas-de-lideranca-de-abraham-lincoln.md</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2335,29 +2449,31 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="b">
-        <v>1</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>2013-06-28</t>
+          <t>2015-01-19</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Saiba como extrair o máximo do comparador de preços Buscapé</t>
+          <t>Por que Anjo?</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>saiba-como-extrair-o-maximo-do-comparador-de-precos-buscape</t>
+          <t>por-que-anjo</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>saiba-como-extrair-o-maximo-do-comparador-de-precos-buscape.md</t>
+          <t>por-que-anjo.md</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2374,29 +2490,31 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="b">
-        <v>1</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2013-06-10</t>
+          <t>2015-01-07</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Universidade Buscapé Company e Endeavor Brasil selam parceria para capacitar empreendedores</t>
+          <t>Empreender é a arte da superação</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>universidade-buscape-company-e-endeavor-brasil-selam-parceria-para-capacitar-empreendedores</t>
+          <t>empreender-e-a-arte-da-superacao</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>universidade-buscape-company-e-endeavor-brasil-selam-parceria-para-capacitar-empreendedores.md</t>
+          <t>empreender-e-a-arte-da-superacao.md</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2413,29 +2531,31 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="b">
-        <v>1</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>2013-05-24</t>
+          <t>2014-12-01</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Como deve ser uma startup?</t>
+          <t>Black Friday 2014 movimenta 1,16 bilhão</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>como-deve-ser-uma-startup</t>
+          <t>black-friday-2014-movimenta-116-bilhao-na-black-friday</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>como-deve-ser-uma-startup.md</t>
+          <t>black-friday-2014-movimenta-116-bilhao-na-black-friday.md</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2452,29 +2572,31 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="b">
-        <v>1</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2013-05-14</t>
+          <t>2014-11-24</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>O mundo da mobilidade</t>
+          <t>Por um choque de inovação no Poder Público</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>o-mundo-da-mobilidade</t>
+          <t>por-um-choque-de-inovacao-no-poder-publico</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>o-mundo-da-mobilidade.md</t>
+          <t>por-um-choque-de-inovacao-no-poder-publico.md</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2491,29 +2613,31 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="b">
-        <v>1</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2013-04-04</t>
+          <t>2014-11-13</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Uma nova tendência chamada Coolhunting</t>
+          <t>Investidor-anjo ou diabo?</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>uma-nova-tendencia-chamada-coolhunting</t>
+          <t>investidor-anjo-ou-diabo</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>uma-nova-tendencia-chamada-coolhunting.md</t>
+          <t>investidor-anjo-ou-diabo.md</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2530,29 +2654,31 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="b">
-        <v>1</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2013-02-22</t>
+          <t>2014-10-15</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>O abandono do carrinho de compras</t>
+          <t>E o empreendedorismo, candidatos?</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>o-abandono-do-carrinho-de-compras</t>
+          <t>e-o-empreendedorismo</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>o-abandono-do-carrinho-de-compras.md</t>
+          <t>e-o-empreendedorismo.md</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2569,29 +2695,31 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="b">
-        <v>1</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2013-02-14</t>
+          <t>2014-09-16</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Tendências do Digital Commerce</t>
+          <t>Seu concorrente está a um dedo de distância</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>tendencias-do-digital-commerce</t>
+          <t>mobilidade-seu-concorrente-esta-a-um-dedo-de-distancia</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>tendencias-do-digital-commerce.md</t>
+          <t>mobilidade-seu-concorrente-esta-a-um-dedo-de-distancia.md</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2608,29 +2736,31 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="b">
-        <v>1</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2013-02-09</t>
+          <t>2014-08-14</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Dicas para levar sua ideia ao sucesso</t>
+          <t>Acredite no impossível! Palestra na Feira do Empreendedor Sebrae</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>dicas-para-levar-sua-ideia-ao-sucesso</t>
+          <t>palestra-na-feira-do-empreendedor-sebrae</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>dicas-para-levar-sua-ideia-ao-sucesso.md</t>
+          <t>palestra-na-feira-do-empreendedor-sebrae.md</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2647,29 +2777,31 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="b">
-        <v>1</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2013-02-08</t>
+          <t>2014-07-28</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Mais um começo</t>
+          <t>10 dicas para você conseguir um bom investidor-anjo</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>mais-um-comeco</t>
+          <t>10-dicas-para-voce-conseguir-um-bom-investidor-anjo</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>mais-um-comeco.md</t>
+          <t>10-dicas-para-voce-conseguir-um-bom-investidor-anjo.md</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2686,29 +2818,31 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="b">
-        <v>1</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2013-02-08</t>
+          <t>2014-06-06</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>A arte de empreender</t>
+          <t>Reflexões de um debutante</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>a-arte-de-empreender</t>
+          <t>reflexoes-de-um-debutante</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>a-arte-de-empreender.md</t>
+          <t>reflexoes-de-um-debutante.md</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2725,29 +2859,31 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="b">
-        <v>1</v>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2013-02-02</t>
+          <t>2014-04-22</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Por uma internet mais segura</t>
+          <t>Manual para um E-commerce B2B de Sucesso</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>por-uma-internet-mais-segura</t>
+          <t>manual-para-um-e-commerce-b2b-de-sucesso</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>por-uma-internet-mais-segura.md</t>
+          <t>manual-para-um-e-commerce-b2b-de-sucesso.md</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2758,6 +2894,744 @@
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2014-03-28</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Tendências para a tecnologia em 2014</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>tendencias-para-a-tecnologia-em-2014</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>tendencias-para-a-tecnologia-em-2014.md</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2014-02-06</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Como usar as redes sociais para atrair talentos para a sua startup</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>como-usar-as-redes-sociais-para-atrair-talentos-para-a-sua-startup</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>como-usar-as-redes-sociais-para-atrair-talentos-para-a-sua-startup.md</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2014-01-28</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Um legado para gestão startup</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>um-legado-para-gestao-startup</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>um-legado-para-gestao-startup.md</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2014-01-10</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Seis dicas para melhorar o perfil no LinkedIn</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>seis-dicas-para-melhorar-o-perfil-no-linkedin</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>seis-dicas-para-melhorar-o-perfil-no-linkedin.md</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>2013-11-14</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Marco Civil, sociedade e mercado digital</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>marco-civil-sociedade-e-mercado-digital</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>marco-civil-sociedade-e-mercado-digital.md</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2013-11-07</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Uma história de sucesso: de uma garagem na Pedroso Alvarenga para o mundo</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>uma-historia-de-sucesso</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>uma-historia-de-sucesso.md</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2013-09-13</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>A Cultura do Fracasso</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>a-cultura-do-fracasso</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>a-cultura-do-fracasso.md</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2013-06-28</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Saiba como extrair o máximo do comparador de preços Buscapé</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>saiba-como-extrair-o-maximo-do-comparador-de-precos-buscape</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>saiba-como-extrair-o-maximo-do-comparador-de-precos-buscape.md</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2013-06-10</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Universidade Buscapé Company e Endeavor Brasil selam parceria para capacitar empreendedores</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>universidade-buscape-company-e-endeavor-brasil-selam-parceria-para-capacitar-empreendedores</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>universidade-buscape-company-e-endeavor-brasil-selam-parceria-para-capacitar-empreendedores.md</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2013-05-24</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Como deve ser uma startup?</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>como-deve-ser-uma-startup</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>como-deve-ser-uma-startup.md</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2013-05-14</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>O mundo da mobilidade</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>o-mundo-da-mobilidade</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>o-mundo-da-mobilidade.md</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2013-04-04</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Uma nova tendência chamada Coolhunting</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>uma-nova-tendencia-chamada-coolhunting</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>uma-nova-tendencia-chamada-coolhunting.md</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2013-02-22</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>O abandono do carrinho de compras</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>o-abandono-do-carrinho-de-compras</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>o-abandono-do-carrinho-de-compras.md</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>2013-02-14</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Tendências do Digital Commerce</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>tendencias-do-digital-commerce</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>tendencias-do-digital-commerce.md</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2013-02-09</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Dicas para levar sua ideia ao sucesso</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>dicas-para-levar-sua-ideia-ao-sucesso</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>dicas-para-levar-sua-ideia-ao-sucesso.md</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2013-02-08</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>A arte de empreender</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>a-arte-de-empreender</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>a-arte-de-empreender.md</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>2013-02-08</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Mais um começo</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>mais-um-comeco</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>mais-um-comeco.md</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Recuperado do blog antigo (Wayback Machine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2013-02-02</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Por uma internet mais segura</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>por-uma-internet-mais-segura</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>por-uma-internet-mais-segura.md</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
         <is>
           <t>Recuperado do blog antigo (Wayback Machine).</t>
         </is>

</xml_diff>

<commit_message>
feat(ideias): /en/ideas não repete texto que já tem versão em inglês na lista
"Boom de fintechs" e "Forças do setor" (LinkedIn, PT) apontam como
versão em inglês para os textos do TechCrunch, que já são linhas da
lista: a /en/ideas mostra só o TechCrunch. Total, description e
ItemList em inglês contam 72.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ideias.xlsx
+++ b/data/ideias.xlsx
@@ -1276,8 +1276,16 @@
           <t>pt</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Brazil’s fintech boom offers new vertical opportunities for investors</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2017/05/13/brazils-fintech-boom-offers-new-vertical-opportunities-for-investors</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>LinkedIn Pulse. Versão em português do texto do TechCrunch de 2017-05-13.</t>
@@ -1399,8 +1407,16 @@
           <t>pt</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Brazil’s tech-sector bright spots beckon as it begins to emerge from long economic crisis</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2016/09/17/brazils-tech-sector-bright-spots-beckon-as-it-begins-to-emerge-from-long-economic-crisis</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>LinkedIn Pulse. Versão em português do texto do TechCrunch de 2016-09-17.</t>

</xml_diff>